<commit_message>
feat: export rule problog, jsonl
</commit_message>
<xml_diff>
--- a/data/processed/ontology/controlled_vocabulary.xlsx
+++ b/data/processed/ontology/controlled_vocabulary.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2614,17 +2614,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>cong_ty_cap_nhat_kip_thoi_thay_doi_co_dong_trong_so_dang_ky_co_dong</t>
+          <t>cong_ty_cap_nhat_kip_thoi_thay_doi_co_dong_trong_so_dang_ky_co_dong_theo_yeu_cau_cua_co_dong_co_lien_quan</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>chuyen_tu_effect:cong_ty_cap_nhat_kip_thoi_thay_doi_co_dong_trong_so_dang_ky_co_dong</t>
+          <t>chuyen_tu_effect:cong_ty_cap_nhat_kip_thoi_thay_doi_co_dong_trong_so_dang_ky_co_dong_theo_yeu_cau_cua_co_dong_co_lien_quan</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `cong_ty_cap_nhat_kip_thoi_thay_doi_co_dong_trong_so_dang_ky_co_dong_theo_yeu_cau_cua_co_dong_co_lien_quan`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `cong_ty_cap_nhat_kip_thoi_thay_doi_co_dong_trong_so_dang_ky_co_dong_theo_yeu_cau_cua_co_dong_co_lien_quan`.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `cong_ty_gui_ve_cong_ty_phieu_lay_y_kien`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `cong_ty_gui_ve_cong_ty_phieu_lay_y_kien`.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `cong_ty_cap_nhat_danh_sach_nhung_nguoi_co_lien_quan_cua_cong_ty`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `cong_ty_cap_nhat_danh_sach_nhung_nguoi_co_lien_quan_cua_cong_ty`.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `co_quan_dang_ky_kinh_doanh_xem_xet_va_cap_giay_chung_nhan_dang_ky_doanh_nghiep`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `co_quan_dang_ky_kinh_doanh_xem_xet_va_cap_giay_chung_nhan_dang_ky_doanh_nghiep`.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `co_quan_dang_ky_kinh_doanh_xem_xet_tinh_hop_le_cua_ho_so_dang_ky_doanh_nghiep_va_cap_dang_ky_doanh_nghiep`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `co_quan_dang_ky_kinh_doanh_xem_xet_tinh_hop_le_cua_ho_so_dang_ky_doanh_nghiep_va_cap_dang_ky_doanh_nghiep`.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `co_quan_dang_ky_kinh_doanh_xem_xet_tinh_hop_le_cua_ho_so_va_cap_giay_chung_nhan_dang_ky_doanh_nghiep_moi`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `co_quan_dang_ky_kinh_doanh_xem_xet_tinh_hop_le_cua_ho_so_va_cap_giay_chung_nhan_dang_ky_doanh_nghiep_moi`.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2896,17 +2896,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>co_quan_dang_ky_kinh_doanh_cap_thong_tin_duoc_luu_giu_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_va_phai_nop_phi</t>
+          <t>duoc_cap_thong_tin_duoc_luu_giu_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_va_phai_nop_phi</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>chuyen_tu_effect:co_quan_dang_ky_kinh_doanh_cap_thong_tin_duoc_luu_giu_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_va_phai_nop_phi</t>
+          <t>chuyen_tu_effect:duoc_cap_thong_tin_duoc_luu_giu_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_va_phai_nop_phi</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `co_quan_dang_ky_kinh_doanh_cap_thong_tin_duoc_luu_giu_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_va_phai_nop_phi`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `duoc_cap_thong_tin_duoc_luu_giu_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_va_phai_nop_phi`.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2943,17 +2943,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>co_quan_dang_ky_kinh_doanh_xem_xet_tinh_hop_le_cua_ho_so_va_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh</t>
+          <t>co_quan_dang_ky_kinh_doanh_cap_thong_tin_duoc_luu_giu_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_va_phai_nop_phi</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>chuyen_tu_effect:co_quan_dang_ky_kinh_doanh_xem_xet_tinh_hop_le_cua_ho_so_va_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh</t>
+          <t>chuyen_tu_effect:co_quan_dang_ky_kinh_doanh_cap_thong_tin_duoc_luu_giu_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_va_phai_nop_phi</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `co_quan_dang_ky_kinh_doanh_xem_xet_tinh_hop_le_cua_ho_so_va_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `co_quan_dang_ky_kinh_doanh_cap_thong_tin_duoc_luu_giu_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_va_phai_nop_phi`.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D45_K3_E000041_H54A3724FA902__05e1c142b45446</t>
+          <t>RULE_LUATDN_D33_K1_E000040_HBD0F2B965340__e0be59d28bca43</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2990,17 +2990,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>cong_ty_cap_nhat_kip_thoi_thay_doi_thanh_vien_trong_so_dang_ky_thanh_vien</t>
+          <t>co_quan_dang_ky_kinh_doanh_xem_xet_tinh_hop_le_cua_ho_so_va_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>chuyen_tu_effect:cong_ty_cap_nhat_kip_thoi_thay_doi_thanh_vien_trong_so_dang_ky_thanh_vien</t>
+          <t>chuyen_tu_effect:co_quan_dang_ky_kinh_doanh_xem_xet_tinh_hop_le_cua_ho_so_va_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `cong_ty_cap_nhat_kip_thoi_thay_doi_thanh_vien_trong_so_dang_ky_thanh_vien_theo_yeu_cau_cua_thanh_vien_co_lien_quan`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `co_quan_dang_ky_kinh_doanh_xem_xet_tinh_hop_le_cua_ho_so_va_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh`.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D48_K3_E000054_H7C5394B2A508__0618df5626c3cd</t>
+          <t>RULE_LUATDN_D45_K3_E000041_H54A3724FA902__05e1c142b45446</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3037,17 +3037,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>cong_ty_gui_phieu_lay_y_kien_ve_cong_ty</t>
+          <t>cong_ty_cap_nhat_kip_thoi_thay_doi_thanh_vien_trong_so_dang_ky_thanh_vien_theo_yeu_cau_cua_thanh_vien_co_lien_quan</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>chuyen_tu_effect:cong_ty_gui_phieu_lay_y_kien_ve_cong_ty</t>
+          <t>chuyen_tu_effect:cong_ty_cap_nhat_kip_thoi_thay_doi_thanh_vien_trong_so_dang_ky_thanh_vien_theo_yeu_cau_cua_thanh_vien_co_lien_quan</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `cong_ty_gui_phieu_lay_y_kien_ve_cong_ty`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `cong_ty_cap_nhat_kip_thoi_thay_doi_thanh_vien_trong_so_dang_ky_thanh_vien_theo_yeu_cau_cua_thanh_vien_co_lien_quan`.</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D61_K3_D_E000058_H55FDA829DADB__3659a9a3d4de76</t>
+          <t>RULE_LUATDN_D48_K3_E000054_H7C5394B2A508__0618df5626c3cd</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3084,17 +3084,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>cong_ty_truoc_hoi_dong_thanh_vien_ve_viec_thuc_hien_quyen_va_nghia_vu_cua_minh</t>
+          <t>cong_ty_gui_phieu_lay_y_kien_ve_cong_ty</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>chuyen_tu_effect:cong_ty_truoc_hoi_dong_thanh_vien_ve_viec_thuc_hien_quyen_va_nghia_vu_cua_minh</t>
+          <t>chuyen_tu_effect:cong_ty_gui_phieu_lay_y_kien_ve_cong_ty</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `cong_ty_truoc_hoi_dong_thanh_vien_ve_viec_thuc_hien_quyen_va_nghia_vu_cua_minh`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `cong_ty_gui_phieu_lay_y_kien_ve_cong_ty`.</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D63_K1_E000063_H87D3F0FBD99C__bad2ab5e0b47d7</t>
+          <t>RULE_LUATDN_D61_K3_D_E000058_H55FDA829DADB__3659a9a3d4de76</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3131,17 +3131,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>co_quan_dang_ky_kinh_doanh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+          <t>cong_ty_truoc_hoi_dong_thanh_vien_ve_viec_thuc_hien_quyen_va_nghia_vu_cua_minh</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>chuyen_tu_effect:co_quan_dang_ky_kinh_doanh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+          <t>chuyen_tu_effect:cong_ty_truoc_hoi_dong_thanh_vien_ve_viec_thuc_hien_quyen_va_nghia_vu_cua_minh</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `co_quan_dang_ky_kinh_doanh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `cong_ty_truoc_hoi_dong_thanh_vien_ve_viec_thuc_hien_quyen_va_nghia_vu_cua_minh`.</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>RULE_ND168_D31_K3_E000266_H1509A1A35C79__4bce78214f31d1; RULE_ND168_D41_K2_E000273_H906A9A038A6C__f824edde05271e; RULE_ND168_D42_K2_E000275_H821D573EEDF4__530e6c2ac4eb1f; RULE_ND168_D43_K5_E000277_H0243FD848FE3__802b6f2206ab87; RULE_ND168_D44_K5_E000279_HCA503CFECDA8__aa2d89008e4cec</t>
+          <t>RULE_LUATDN_D63_K1_E000063_H87D3F0FBD99C__bad2ab5e0b47d7</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3178,17 +3178,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>co_quan_dang_ky_kinh_doanh_cap_tinh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+          <t>chap_thuan_thi_co_quan_dang_ky_kinh_doanh_cap_xa_ra_quyet_dinh_thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_trong_thoi_han_03_ngay_lam_viec_ke_tu_ngay_ket_thuc_thoi_han</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>chuyen_tu_effect:co_quan_dang_ky_kinh_doanh_cap_tinh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+          <t>chuyen_tu_effect:chap_thuan_thi_co_quan_dang_ky_kinh_doanh_cap_xa_ra_quyet_dinh_thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_trong_thoi_han_03_ngay_lam_viec_ke_tu_ngay_ket_thuc_thoi_han</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `co_quan_dang_ky_kinh_doanh_cap_tinh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so`.</t>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `chap_thuan_thi_co_quan_dang_ky_kinh_doanh_cap_xa_ra_quyet_dinh_thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_trong_thoi_han_03_ngay_lam_viec_ke_tu_ngay_ket_thuc_thoi_han`.</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>RULE_ND168_D31_K3_E000415_HF96DE9D9BF08__715810e59d4772; RULE_ND168_D41_K2_E000425_HEEADD79DF7E1__341dcc712fe43d; RULE_ND168_D42_K2_E000430_H871CDC7A0EBD__6112b7ae8b0e38; RULE_ND168_D43_K5_E000435_HADF045408BC9__6a55deefc5885c; RULE_ND168_D44_K5_E000440_H3776FA482E45__895dd1b8852a0c</t>
+          <t>RULE_ND168_D107_K4_E000323_HC7780C522732__8b02a06325d0fb; RULE_ND168_D107_K4_E000503_HAD9534ACA4E3__80fbe079a9ef2a</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3225,40 +3225,228 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
+          <t>co_quan_dang_ky_kinh_doanh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>chuyen_tu_effect:co_quan_dang_ky_kinh_doanh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `co_quan_dang_ky_kinh_doanh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so`.</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>mapping_hanh_vi_khong_phai_ket_qua</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>RULE_ND168_D31_K3_E000266_H1509A1A35C79__4bce78214f31d1; RULE_ND168_D41_K2_E000273_H906A9A038A6C__f824edde05271e; RULE_ND168_D42_K2_E000275_H821D573EEDF4__530e6c2ac4eb1f; RULE_ND168_D43_K5_E000277_H0243FD848FE3__802b6f2206ab87; RULE_ND168_D44_K5_E000279_HCA503CFECDA8__aa2d89008e4cec</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>trung_binh</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>chuyen_action_ra_khoi_effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>hanh_vi</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>co_quan_dang_ky_kinh_doanh_cap_tinh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>chuyen_tu_effect:co_quan_dang_ky_kinh_doanh_cap_tinh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `co_quan_dang_ky_kinh_doanh_cap_tinh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so`.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>mapping_hanh_vi_khong_phai_ket_qua</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>RULE_ND168_D31_K3_E000415_HF96DE9D9BF08__715810e59d4772; RULE_ND168_D41_K2_E000425_HEEADD79DF7E1__341dcc712fe43d; RULE_ND168_D42_K2_E000430_H871CDC7A0EBD__6112b7ae8b0e38; RULE_ND168_D43_K5_E000435_HADF045408BC9__6a55deefc5885c; RULE_ND168_D44_K5_E000440_H3776FA482E45__895dd1b8852a0c</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>trung_binh</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>chuyen_action_ra_khoi_effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>hanh_vi</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
           <t>nguoi_thanh_lap_doanh_nghiep_thuc_hien_day_du</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>chuyen_tu_effect:nguoi_thanh_lap_doanh_nghiep_thuc_hien_day_du</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). Gốc: `nguoi_thanh_lap_doanh_nghiep_thuc_hien_day_du`.</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `nguoi_thanh_lap_doanh_nghiep_thuc_hien_day_du`.</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>mapping_hanh_vi_khong_phai_ket_qua</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>RULE_ND168_D5_K2_E000197_HA0ABBF5F3EF2__802411e0d0015e</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G67" t="inlineStr">
         <is>
           <t>co</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="H67" t="inlineStr">
         <is>
           <t>trung_binh</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>chuyen_action_ra_khoi_effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>hanh_vi</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>cham_dut_hoat_dong_chi_nhanh_doanh_nghiep_phai_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_c</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>chuyen_tu_effect:cham_dut_hoat_dong_chi_nhanh_doanh_nghiep_phai_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_c</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `cham_dut_hoat_dong_chi_nhanh_doanh_nghiep_phai_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_c`.</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>mapping_hanh_vi_khong_phai_ket_qua</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>RULE_ND168_D66_K5_E000304_HF34F2F907D78__50796ed7bced1b; RULE_ND168_D66_K5_E000483_H87A2DB73760C__e6f80f3364ef77</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>trung_binh</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>chuyen_action_ra_khoi_effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>hanh_vi</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>cham_dut_hoat_dong_chi_nhanh_doanh_nghiep_phai_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan_dang_ky_kinh_doanh_cap_tinh_noi_dat_dia</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>chuyen_tu_effect:cham_dut_hoat_dong_chi_nhanh_doanh_nghiep_phai_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan_dang_ky_kinh_doanh_cap_tinh_noi_dat_dia</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Diễn đạt hành vi/thủ tục (đưa khỏi effect). `cham_dut_hoat_dong_chi_nhanh_doanh_nghiep_phai_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan_dang_ky_kinh_doanh_cap_tinh</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>mapping_hanh_vi_khong_phai_ket_qua</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>RULE_ND168_D66_K5_E000482_H87A2DB73760C__0abeaa88313a85</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>co</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>trung_binh</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
         <is>
           <t>chuyen_action_ra_khoi_effect</t>
         </is>
@@ -3323,7 +3511,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3356,16 +3544,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3398,11 +3582,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3440,11 +3620,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3482,11 +3658,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3524,11 +3696,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3566,16 +3734,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>giao_dich</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3608,16 +3772,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>giao_dich</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3650,11 +3810,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3692,11 +3848,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3734,16 +3886,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>nghia_vu_tai_san</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3776,11 +3924,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3818,11 +3962,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3860,16 +4000,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3902,11 +4038,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3944,16 +4076,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>giao_dich</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3986,11 +4114,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4028,11 +4152,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4070,16 +4190,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4112,16 +4228,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4154,11 +4266,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4196,16 +4304,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4238,16 +4342,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4280,16 +4380,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>thong_tin</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4322,11 +4418,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4364,16 +4456,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4406,16 +4494,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>co_phan_thanh_vien</t>
+          <t>thanh_vien</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4448,11 +4532,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4490,11 +4570,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4532,16 +4608,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>co_phan_thanh_vien</t>
+          <t>thanh_vien</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4574,11 +4646,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4616,16 +4684,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>von_gop_von</t>
+          <t>von</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4658,11 +4722,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4700,11 +4760,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4742,16 +4798,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4784,11 +4836,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4826,16 +4874,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4868,11 +4912,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4910,16 +4950,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4952,16 +4988,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4994,16 +5026,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -5036,11 +5064,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5078,16 +5102,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5120,16 +5140,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5162,16 +5178,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5204,16 +5216,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5246,16 +5254,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5288,16 +5292,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5330,16 +5330,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5372,16 +5368,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5414,16 +5406,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -5456,16 +5444,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -5498,16 +5482,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -5540,16 +5520,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -5582,16 +5558,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -5624,16 +5596,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -5666,16 +5634,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -5708,11 +5672,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5750,16 +5710,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -5792,16 +5748,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -5834,16 +5786,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>von</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -5876,16 +5824,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5918,16 +5862,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>thong_tin</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -5960,16 +5900,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -6002,16 +5938,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -6044,16 +5976,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -6086,16 +6014,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -6128,11 +6052,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6170,11 +6090,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6212,16 +6128,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -6254,16 +6166,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -6296,16 +6204,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -6338,16 +6242,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -6380,16 +6280,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -6422,16 +6318,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -6464,16 +6356,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -6506,16 +6394,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>giay_chung_nhan</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -6548,16 +6432,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>ho_so</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -6590,16 +6470,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>noi_dung_dang_ky</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -6632,11 +6508,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6674,11 +6546,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6716,16 +6584,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>noi_dung_dang_ky</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -6758,16 +6622,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -6800,16 +6660,12 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ho_so_tai_lieu</t>
+          <t>danh_sach</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -6842,11 +6698,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H85" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6859,7 +6711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6940,11 +6792,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6982,11 +6830,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7024,11 +6868,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7066,11 +6906,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7108,11 +6944,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7150,11 +6982,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7234,11 +7062,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7276,11 +7100,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7318,11 +7138,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7360,11 +7176,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7402,11 +7214,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7444,11 +7252,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7486,11 +7290,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7528,11 +7328,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7570,11 +7366,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7612,11 +7404,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7631,7 +7419,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>chấm dứt hoạt động</t>
+          <t>chấm dứt hoạt động đối với chi nhánh; văn phòng đại diện; địa điểm kinh doanh; chấm dứt hoạt động</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -7641,22 +7429,22 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>RULE_ND168_D27_K3_B_E000408_H645CC4278C14__726aecd2fd98e0</t>
+          <t>RULE_ND168_D118_K3_E000522_H0811C24751E0__7fb44d85940b04; RULE_ND168_D118_K3_E000341_H6839229D9C6F__6f008278ee22c6; RULE_ND168_D27_K3_B_E000408_H645CC4278C14__726aecd2fd98e0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>cao</t>
+          <t>trung_binh</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>tach_condition_khoi_effect</t>
         </is>
       </c>
     </row>
@@ -7668,22 +7456,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>cham_dut_hoat_dong_chi_nhanh_doanh_nghiep_phai_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_c</t>
+          <t>cham_dut_hoat_dong_chiu_trach_nhiem_thuc_hien_cac_hop_dong_thanh_toan_cac_khoan_no_gom_ca_no_thue_cua_chi_nhanh_va_t</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>chấm dứt hoạt động chi nhánh, doanh nghiệp phải thực hiện thủ tục chấm dứt hoạt động của tất cả địa điểm kinh doanh trực thuộc c</t>
+          <t>chấm dứt hoạt động chịu trách nhiệm thực hiện các hợp đồng, thanh toán các khoản nợ, gồm cả nợ thuế của chi nhánh và t</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_chi_nhanh_doanh_nghiep_phai_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_c`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_chiu_trach_nhiem_thuc_hien_cac_hop_dong_thanh_toan_cac_khoan_no_gom_ca_no_thue_cua_chi_nhanh_va_t`.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RULE_ND168_D66_K5_E000304_HF34F2F907D78__50796ed7bced1b; RULE_ND168_D66_K5_E000483_H87A2DB73760C__e6f80f3364ef77</t>
+          <t>RULE_LUATDN_D213_K3_E000191_HF074DD2CC305__cd4b8a1e04da78</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -7696,11 +7484,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7710,22 +7494,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>cham_dut_hoat_dong_chi_nhanh_doanh_nghiep_phai_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan_dang_ky_kinh_doanh_cap_tinh_noi_dat_dia</t>
+          <t>cham_dut_hoat_dong_chiu_trach_nhiem_thuc_hien_cac_hop_dong_thanh_toan_cac_khoan_no_gom_ca_no_thue_cua_chi_nhanh_va_tiep_tuc_su_dung_lao_dong_hoac_giai_quyet_du_quyen_loi_hop_phap_cho_ngu</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>chấm dứt hoạt động chi nhánh, doanh nghiệp phải thực hiện thủ tục chấm dứt hoạt động của tất cả địa điểm kinh doanh trực thuộc chi nhánh tại Cơ quan đăng ký kinh doanh cấp tỉnh nơi đặt địa</t>
+          <t>chấm dứt hoạt động chịu trách nhiệm thực hiện các hợp đồng, thanh toán các khoản nợ, gồm cả nợ thuế của chi nhánh và tiếp tục sử dụng lao động hoặc giải quyết đủ quyền lợi hợp pháp cho ngư</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_chi_nhanh_doanh_nghiep_phai_thuc_hien_thu_tuc_cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan_dang_ky_kinh_doanh_cap_tinh_noi_dat_di</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_chiu_trach_nhiem_thuc_hien_cac_hop_dong_thanh_toan_cac_khoan_no_gom_ca_no_thue_cua_chi_nhanh_va_tiep_tuc_su_dung_lao_dong_hoac_giai_quyet_du_quyen_loi_hop_phap_cho_ngu</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>RULE_ND168_D66_K5_E000482_H87A2DB73760C__0abeaa88313a85</t>
+          <t>RULE_LUATDN_D213_K3_E000380_H8F80CAF77D48__c1b4b55e3b1389; RULE_LUATDN_D213_K3_E000189_HF074DD2CC305__1bbabbdbe86f35</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -7738,11 +7522,7 @@
           <t>trung_binh</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7752,22 +7532,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>cham_dut_hoat_dong_chiu_trach_nhiem_thuc_hien_cac_hop_dong_thanh_toan_cac_khoan_no_gom_ca_no_thue_cua_chi_nhanh_va_t</t>
+          <t>cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan_dang_ky_kinh_doanh</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>chấm dứt hoạt động chịu trách nhiệm thực hiện các hợp đồng, thanh toán các khoản nợ, gồm cả nợ thuế của chi nhánh và t</t>
+          <t>chấm dứt hoạt động của tất cả địa điểm kinh doanh trực thuộc chi nhánh tại Cơ quan đăng ký kinh doanh</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_chiu_trach_nhiem_thuc_hien_cac_hop_dong_thanh_toan_cac_khoan_no_gom_ca_no_thue_cua_chi_nhanh_va_t`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan_dang_ky_kinh_doanh`.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D213_K3_E000191_HF074DD2CC305__cd4b8a1e04da78</t>
+          <t>RULE_ND168_D66_K5_E000303_HF34F2F907D78__8430406cf71e7d</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -7780,11 +7560,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7794,22 +7570,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>cham_dut_hoat_dong_chiu_trach_nhiem_thuc_hien_cac_hop_dong_thanh_toan_cac_khoan_no_gom_ca_no_thue_cua_chi_nhanh_va_tiep_tuc_su_dung_lao_dong_hoac_giai_quyet_du_quyen_loi_hop_phap_cho_ngu</t>
+          <t>cham_dut_hoat_dong_trong_co_so_du_lieu_ve_dang_ky_ho_kinh_doanh</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>chấm dứt hoạt động chịu trách nhiệm thực hiện các hợp đồng, thanh toán các khoản nợ, gồm cả nợ thuế của chi nhánh và tiếp tục sử dụng lao động hoặc giải quyết đủ quyền lợi hợp pháp cho ngư</t>
+          <t>chấm dứt hoạt động trong Cơ sở dữ liệu về đăng ký hộ kinh doanh</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_chiu_trach_nhiem_thuc_hien_cac_hop_dong_thanh_toan_cac_khoan_no_gom_ca_no_thue_cua_chi_nhanh_va_tiep_tuc_su_dung_lao_dong_hoac_giai_quyet_du_quyen_loi_hop_phap_cho_ngu</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_trong_co_so_du_lieu_ve_dang_ky_ho_kinh_doanh`.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D213_K3_E000380_H8F80CAF77D48__c1b4b55e3b1389; RULE_LUATDN_D213_K3_E000189_HF074DD2CC305__1bbabbdbe86f35</t>
+          <t>RULE_ND168_D27_K3_B_E000407_H645CC4278C14__48dee7f15d2346</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -7819,39 +7595,35 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>trung_binh</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>cao</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cham_dut</t>
+          <t>chap_thuan</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>cham_dut_hoat_dong_cua_ho_kinh_doanh_cho_co_quan_thue_va_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut</t>
+          <t>chap_thuan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>chấm dứt hoạt động của hộ kinh doanh cho Cơ quan thuế và ra thông báo về việc hộ kinh doanh đang làm thủ tục chấm dứt</t>
+          <t>chấp thuận; trừ trường hợp Hội đồng thành viên quyết định thời hạn khác</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_cua_ho_kinh_doanh_cho_co_quan_thue_va_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `chap_thuan`.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>RULE_ND168_D27_K3_B_E000406_H645CC4278C14__ca5b42fe13202c</t>
+          <t>RULE_LUATDN_D186_K1_E000124_HFF0DAB317E93__e594e48a541eab; RULE_ND168_D59_K2_B_E000479_H6CE5F7A93C8B__e80d74b1b90e68; RULE_ND168_D59_K2_B_E000301_HB765E274CC42__e48ea797ee3048; RULE_LUATDN_D186_K2_E000128_H978952EE6FD4__271a076b3bf9cb; RULE_LUATDN_D186_K2_E000364_HC305BFE2E363__e1e8bea05ff736; RULE_LUATDN_D186_K2_E000125_H2FC30FD46A92__59df9f03b09822</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -7866,34 +7638,34 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>tach_exception_khoi_effect</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>cham_dut</t>
+          <t>chap_thuan</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>cham_dut_hoat_dong_cua_ho_kinh_doanh_cho_co_quan_thue_va_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_tren_cong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_chuyen</t>
+          <t>chap_thuan_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>chấm dứt hoạt động của hộ kinh doanh cho Cơ quan thuế và ra thông báo về việc hộ kinh doanh đang làm thủ tục chấm dứt hoạt động trên Cổng thông tin quốc gia về đăng ký doanh nghiệp, chuyển</t>
+          <t>chấp thuận trên Hệ thống thông tin quốc gia về đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_cua_ho_kinh_doanh_cho_co_quan_thue_va_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_tren_cong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_chuye</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `chap_thuan_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep`.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>RULE_ND168_D27_K3_B_E000405_H645CC4278C14__2da370c26df78e</t>
+          <t>RULE_ND168_D31_K6_E000267_H565D1BB5E0AC__243ed69455d8ce; RULE_ND168_D31_K6_E000271_H565D1BB5E0AC__515f331279a5a7; RULE_ND168_D31_K6_E000416_HF58B712D1CE4__7867763b848ee0; RULE_ND168_D31_K6_E000419_H46A4A566E7A4__38e6cb2ba88b0e</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -7903,39 +7675,35 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>trung_binh</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+          <t>cao</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>cham_dut</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan_dang_ky_kinh_doanh</t>
+          <t>co_quan_dang_ky_kinh_doanh_ap_dung_quy_dinh_loai_tru</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>chấm dứt hoạt động của tất cả địa điểm kinh doanh trực thuộc chi nhánh tại Cơ quan đăng ký kinh doanh</t>
+          <t>Cơ quan đăng ký kinh doanh áp dụng quy định loại trừ</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_cua_tat_ca_dia_diem_kinh_doanh_truc_thuoc_chi_nhanh_tai_co_quan_dang_ky_kinh_doanh`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `co_quan_dang_ky_kinh_doanh_ap_dung_quy_dinh_loai_tru`.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>RULE_ND168_D66_K5_E000303_HF34F2F907D78__8430406cf71e7d</t>
+          <t>RULE_ND168_D20_K1_A_E000232_HEBA6CEE992E3__33783bcc8ca8c9</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -7948,36 +7716,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>cham_dut</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>cham_dut_hoat_dong_doi_voi_chi_nhanh_van_phong_dai_dien_dia_diem_kinh_doanh</t>
+          <t>co_quan_dang_ky_kinh_doanh_cap_dang_ky_doanh_nghiep_theo_quy_trinh_du_phong</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>chấm dứt hoạt động đối với chi nhánh, văn phòng đại diện, địa điểm kinh doanh</t>
+          <t>Cơ quan đăng ký kinh doanh cấp đăng ký doanh nghiệp theo quy trình dự phòng</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_doi_voi_chi_nhanh_van_phong_dai_dien_dia_diem_kinh_doanh`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `co_quan_dang_ky_kinh_doanh_cap_dang_ky_doanh_nghiep_theo_quy_trinh_du_phong`.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>RULE_ND168_D118_K3_E000522_H0811C24751E0__7fb44d85940b04; RULE_ND168_D118_K3_E000341_H6839229D9C6F__6f008278ee22c6</t>
+          <t>RULE_ND168_D13_K4_E000222_H7575F6E0A298__e3b2e7405f1543</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -7990,36 +7754,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>cham_dut</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>cham_dut_hoat_dong_trong_co_so_du_lieu_ve_dang_ky_ho_kinh_doanh</t>
+          <t>co_quan_dang_ky_kinh_doanh_cap_tinh_thuc_hien_quan_ly_nha_nuoc</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>chấm dứt hoạt động trong Cơ sở dữ liệu về đăng ký hộ kinh doanh</t>
+          <t>Cơ quan đăng ký kinh doanh cấp tỉnh thực hiện quản lý nhà nước</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `cham_dut_hoat_dong_trong_co_so_du_lieu_ve_dang_ky_ho_kinh_doanh`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `co_quan_dang_ky_kinh_doanh_cap_tinh_thuc_hien_quan_ly_nha_nuoc`.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>RULE_ND168_D27_K3_B_E000407_H645CC4278C14__48dee7f15d2346</t>
+          <t>RULE_LUATDN_D215_K2_E000192_HA15EAD4E7536__4a0d8250bffec5</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -8032,36 +7792,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>chap_thuan</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>chap_thuan</t>
+          <t>co_quan_dang_ky_kinh_doanh_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>chấp thuận</t>
+          <t>Cơ quan đăng ký kinh doanh đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `chap_thuan`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `co_quan_dang_ky_kinh_doanh_dang_ky_doanh_nghiep`.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D186_K1_E000124_HFF0DAB317E93__e594e48a541eab; RULE_ND168_D59_K2_B_E000479_H6CE5F7A93C8B__e80d74b1b90e68; RULE_ND168_D59_K2_B_E000301_HB765E274CC42__e48ea797ee3048</t>
+          <t>RULE_ND168_D20_K1_A_E000234_H8752DA9084F2__4600286e438dc3; RULE_ND168_D20_K1_A_E000230_HA78F4CA68C80__0e0c127de64957</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -8074,120 +7830,108 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>thu_hoi</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>chap_thuan_thi_co_quan_dang_ky_kinh_doanh_cap_tinh_ra_quyet_dinh_thu_hoi_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh_van_phong_dai_dien</t>
+          <t>co_quan_dang_ky_kinh_doanh_thanh_phan_ho_so</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>chấp thuận thì Cơ quan đăng ký kinh doanh cấp tỉnh ra quyết định thu hồi Giấy chứng nhận đăng ký hoạt động chi nhánh, văn phòng đại diện trong thời hạn 03 ngày làm việc k</t>
+          <t>Cơ quan đăng ký kinh doanh thành phần hồ sơ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `chap_thuan_thi_co_quan_dang_ky_kinh_doanh_cap_tinh_ra_quyet_dinh_thu_hoi_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh_van_phong_dai_dien`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `co_quan_dang_ky_kinh_doanh_thanh_phan_ho_so`.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>RULE_ND168_D71_K3_E000497_HD4B75A6952A5__7fe9ff563fe49f</t>
+          <t>RULE_ND168_D15_K4_E000226_H77B8473A5144__f4a8cfe63d7a31</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>trung_binh</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>tach_condition_khoi_effect</t>
-        </is>
-      </c>
+          <t>cao</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>thu_hoi</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>chap_thuan_thi_co_quan_dang_ky_kinh_doanh_cap_xa_ra_quyet_dinh_thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh</t>
+          <t>doanh_nghiep_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>chấp thuận thì Cơ quan đăng ký kinh doanh cấp xã ra quyết định thu hồi Giấy chứng nhận đăng ký hộ kinh doanh trong thời hạn 03 ngày làm việc kể từ ngày kết thúc thời hạn</t>
+          <t>Doanh nghiệp đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `chap_thuan_thi_co_quan_dang_ky_kinh_doanh_cap_xa_ra_quyet_dinh_thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `doanh_nghiep_dang_ky_doanh_nghiep`.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>RULE_ND168_D107_K4_E000323_HC7780C522732__8b02a06325d0fb; RULE_ND168_D107_K4_E000503_HAD9534ACA4E3__80fbe079a9ef2a</t>
+          <t>RULE_ND168_D23_K1_K_E000238_H9F0055EDAC32__8b171c4fe8e666; RULE_ND168_D4_K5_E000194_H71B013782AB6__fe65a55a4c30bb</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>co</t>
+          <t>khong</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>trung_binh</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>tach_condition_khoi_effect</t>
-        </is>
-      </c>
+          <t>cao</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>chap_thuan</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>chap_thuan_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep</t>
+          <t>doanh_nghiep_dang_ky_doanh_nghiep_va_cac_bao_cao</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>chấp thuận trên Hệ thống thông tin quốc gia về đăng ký doanh nghiệp</t>
+          <t>Doanh nghiệp đăng ký doanh nghiệp và các báo cáo</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `chap_thuan_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `doanh_nghiep_dang_ky_doanh_nghiep_va_cac_bao_cao`.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>RULE_ND168_D31_K6_E000267_H565D1BB5E0AC__243ed69455d8ce; RULE_ND168_D31_K6_E000271_H565D1BB5E0AC__515f331279a5a7; RULE_ND168_D31_K6_E000416_HF58B712D1CE4__7867763b848ee0; RULE_ND168_D31_K6_E000419_H46A4A566E7A4__38e6cb2ba88b0e</t>
+          <t>RULE_LUATDN_D8_K3_E000001_H5745E238E6BA__19b1296ca4aca4</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -8200,36 +7944,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>chap_thuan</t>
+          <t>khac</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>chap_thuan_tru_truong_hop_hoi_dong_thanh_vien_quyet_dinh_thoi_han_khac</t>
+          <t>doanh_nghiep_dang_ky_thay_doi_chu_doanh_nghiep_tu_nhan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>chấp thuận, trừ trường hợp Hội đồng thành viên quyết định thời hạn khác</t>
+          <t>Doanh nghiệp đăng ký thay đổi chủ doanh nghiệp tư nhân</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `chap_thuan_tru_truong_hop_hoi_dong_thanh_vien_quyet_dinh_thoi_han_khac`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `doanh_nghiep_dang_ky_thay_doi_chu_doanh_nghiep_tu_nhan`.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D186_K2_E000128_H978952EE6FD4__271a076b3bf9cb; RULE_LUATDN_D186_K2_E000364_HC305BFE2E363__e1e8bea05ff736; RULE_LUATDN_D186_K2_E000125_H2FC30FD46A92__59df9f03b09822</t>
+          <t>RULE_LUATDN_D192_K4_E000143_HDD7294EC5093__a1844b762d174d</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -8242,11 +7982,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8256,22 +7992,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>co_quan_dang_ky_kinh_doanh_ap_dung_quy_dinh_loai_tru</t>
+          <t>doanh_nghiep_nop_du_so_thue</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Cơ quan đăng ký kinh doanh áp dụng quy định loại trừ</t>
+          <t>Doanh nghiệp nộp đủ số thuế</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `co_quan_dang_ky_kinh_doanh_ap_dung_quy_dinh_loai_tru`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `doanh_nghiep_nop_du_so_thue`.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>RULE_ND168_D20_K1_A_E000232_HEBA6CEE992E3__33783bcc8ca8c9</t>
+          <t>RULE_LUATDN_D206_K3_E000182_HB3760B0CD551__0c3013b06a8c7b</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -8284,36 +8020,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>co_quan_dang_ky_kinh_doanh_cap_dang_ky_doanh_nghiep_theo_quy_trinh_du_phong</t>
+          <t>duoc_cap_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Cơ quan đăng ký kinh doanh cấp đăng ký doanh nghiệp theo quy trình dự phòng</t>
+          <t>Được cấp đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `co_quan_dang_ky_kinh_doanh_cap_dang_ky_doanh_nghiep_theo_quy_trinh_du_phong`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_dang_ky_doanh_nghiep`.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>RULE_ND168_D13_K4_E000222_H7575F6E0A298__e3b2e7405f1543</t>
+          <t>RULE_LUATDN_D26_K5_E000011_H3FEBB093524B__f0e073146941eb</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -8326,36 +8058,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>co_quan_dang_ky_kinh_doanh_cap_tinh_thuc_hien_quan_ly_nha_nuoc</t>
+          <t>duoc_cap_dang_ky_doanh_nghiep_theo_quy_trinh_du_phong</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Cơ quan đăng ký kinh doanh cấp tỉnh thực hiện quản lý nhà nước</t>
+          <t>Được cấp đăng ký doanh nghiệp theo quy trình dự phòng</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `co_quan_dang_ky_kinh_doanh_cap_tinh_thuc_hien_quan_ly_nha_nuoc`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_dang_ky_doanh_nghiep_theo_quy_trinh_du_phong`.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D215_K2_E000192_HA15EAD4E7536__4a0d8250bffec5</t>
+          <t>RULE_ND168_D13_K4_E000222_H7575F6E0A298__e3b2e7405f1543</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -8368,36 +8096,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>co_quan_dang_ky_kinh_doanh_dang_ky_doanh_nghiep</t>
+          <t>duoc_cap_giay_chung_nhan_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Cơ quan đăng ký kinh doanh đăng ký doanh nghiệp</t>
+          <t>Được cấp Giấy chứng nhận đăng ký doanh nghiệp | được cấp Giấy chứng nhận đăng ký doanh nghiệp; được cấp Giấy chứng nhận đăng ký doanh nghiệp; trừ trường hợp Điều lệ công ty hoặc hợp đồng đăng ký mua cổ phần quy định một thời hạn khác ngắn hơn</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `co_quan_dang_ky_kinh_doanh_dang_ky_doanh_nghiep`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_giay_chung_nhan_dang_ky_doanh_nghiep`.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>RULE_ND168_D20_K1_A_E000234_H8752DA9084F2__4600286e438dc3; RULE_ND168_D20_K1_A_E000230_HA78F4CA68C80__0e0c127de64957</t>
+          <t>RULE_LUATDN_D113_K1_E000094_HC863DA3A8CBE__234d9c7caeb7b4; RULE_LUATDN_D113_K1_E000085_HABFC666433B3__22c2142f7ac83a; RULE_LUATDN_D113_K1_E000078_H67FF516B0336__96d8cf793c1519; RULE_LUATDN_D205_K2_E000180_HA8EFB2670117__32e45121578765; RULE_LUATDN_D113_K1_E000082_H67FF516B0336__b18dfb4fdee692; RULE_LUATDN_D113_K1_E000083_H4135AC48C5CC__92ac27f8e80f5c; RULE_LUATDN_D113_K1_E000361_H9559D7A7E175__e7c07124cb07f1</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -8412,34 +8136,34 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>tach_exception_khoi_effect</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>co_quan_dang_ky_kinh_doanh_thanh_phan_ho_so</t>
+          <t>duoc_cap_giay_chung_nhan_dang_ky_doanh_nghiep_moi</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Cơ quan đăng ký kinh doanh thành phần hồ sơ</t>
+          <t>Được cấp Giấy chứng nhận đăng ký doanh nghiệp mới</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `co_quan_dang_ky_kinh_doanh_thanh_phan_ho_so`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_giay_chung_nhan_dang_ky_doanh_nghiep_moi`.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>RULE_ND168_D15_K4_E000226_H77B8473A5144__f4a8cfe63d7a31</t>
+          <t>RULE_LUATDN_D30_K3_E000031_H683D2BEC0D69__9f7fb709427928</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -8452,36 +8176,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>doanh_nghiep_dang_ky_doanh_nghiep</t>
+          <t>duoc_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Doanh nghiệp đăng ký doanh nghiệp</t>
+          <t>Được cấp Giấy chứng nhận đăng ký hoạt động chi nhánh</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `doanh_nghiep_dang_ky_doanh_nghiep`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh`.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>RULE_ND168_D23_K1_K_E000238_H9F0055EDAC32__8b171c4fe8e666; RULE_ND168_D4_K5_E000194_H71B013782AB6__fe65a55a4c30bb</t>
+          <t>RULE_LUATDN_D45_K3_E000041_H54A3724FA902__05e1c142b45446</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -8494,36 +8214,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>doanh_nghiep_dang_ky_doanh_nghiep_va_cac_bao_cao</t>
+          <t>duoc_cap_tinh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Doanh nghiệp đăng ký doanh nghiệp và các báo cáo</t>
+          <t>Được cấp tỉnh cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả cho người nộp hồ sơ</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `doanh_nghiep_dang_ky_doanh_nghiep_va_cac_bao_cao`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_tinh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so`.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D8_K3_E000001_H5745E238E6BA__19b1296ca4aca4</t>
+          <t>RULE_ND168_D31_K3_E000415_HF96DE9D9BF08__715810e59d4772; RULE_ND168_D41_K2_E000425_HEEADD79DF7E1__341dcc712fe43d; RULE_ND168_D42_K2_E000430_H871CDC7A0EBD__6112b7ae8b0e38; RULE_ND168_D43_K5_E000435_HADF045408BC9__6a55deefc5885c; RULE_ND168_D44_K5_E000440_H3776FA482E45__895dd1b8852a0c</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -8536,36 +8252,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>doanh_nghiep_dang_ky_thay_doi_chu_doanh_nghiep_tu_nhan</t>
+          <t>duoc_cap_tinh_thuc_hien_quan_ly_nha_nuoc</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Doanh nghiệp đăng ký thay đổi chủ doanh nghiệp tư nhân</t>
+          <t>Được cấp tỉnh thực hiện quản lý nhà nước</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `doanh_nghiep_dang_ky_thay_doi_chu_doanh_nghiep_tu_nhan`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_tinh_thuc_hien_quan_ly_nha_nuoc`.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D192_K4_E000143_HDD7294EC5093__a1844b762d174d</t>
+          <t>RULE_LUATDN_D215_K2_E000192_HA15EAD4E7536__4a0d8250bffec5</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -8578,36 +8290,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>khac</t>
+          <t>cap_giay</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>doanh_nghiep_nop_du_so_thue</t>
+          <t>duoc_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Doanh nghiệp nộp đủ số thuế</t>
+          <t>Được cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả cho người nộp hồ sơ</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `doanh_nghiep_nop_du_so_thue`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so`.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D206_K3_E000182_HB3760B0CD551__0c3013b06a8c7b</t>
+          <t>RULE_ND168_D31_K3_E000266_H1509A1A35C79__4bce78214f31d1; RULE_ND168_D41_K2_E000273_H906A9A038A6C__f824edde05271e; RULE_ND168_D42_K2_E000275_H821D573EEDF4__530e6c2ac4eb1f; RULE_ND168_D43_K5_E000277_H0243FD848FE3__802b6f2206ab87; RULE_ND168_D44_K5_E000279_HCA503CFECDA8__aa2d89008e4cec</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -8620,36 +8328,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>cap_nhat</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>duoc_cap_dang_ky_doanh_nghiep</t>
+          <t>khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_dong_thoi_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_chi_nhanh_van_phong_dai</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Được cấp đăng ký doanh nghiệp</t>
+          <t>khôi phục Giấy chứng nhận đăng ký doanh nghiệp, đồng thời cập nhật tình trạng pháp lý của doanh nghiệp, chi nhánh, văn phòng đại</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_dang_ky_doanh_nghiep`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_dong_thoi_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_chi_nhanh_van_phong_dai`.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D26_K5_E000011_H3FEBB093524B__f0e073146941eb</t>
+          <t>RULE_ND168_D70_K2_E000315_H76391FA4DF19__fd8923adabc565</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -8662,36 +8366,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>cap_nhat</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>duoc_cap_dang_ky_doanh_nghiep_theo_quy_trinh_du_phong</t>
+          <t>khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_dong_thoi_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_chi_nhanh_van_phong_dai_dien_dia_diem_kinh_doanh_trong_co_so_du</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Được cấp đăng ký doanh nghiệp theo quy trình dự phòng</t>
+          <t>khôi phục Giấy chứng nhận đăng ký doanh nghiệp, đồng thời cập nhật tình trạng pháp lý của doanh nghiệp, chi nhánh, văn phòng đại diện, địa điểm kinh doanh trong Cơ sở dữ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_dang_ky_doanh_nghiep_theo_quy_trinh_du_phong`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_dong_thoi_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_chi_nhanh_van_phong_dai_dien_dia_diem_kinh_doanh_trong_co_so_du`.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>RULE_ND168_D13_K4_E000222_H7575F6E0A298__e3b2e7405f1543</t>
+          <t>RULE_ND168_D70_K2_E000490_H294525A8FA40__1aeefc8cc68ed5</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -8704,36 +8404,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>duoc_cap_giay_chung_nhan_dang_ky_doanh_nghiep</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Được cấp Giấy chứng nhận đăng ký doanh nghiệp | được cấp Giấy chứng nhận đăng ký doanh nghiệp; được cấp Giấy chứng nhận đăng ký doanh nghiệp; trừ trường hợp Điều lệ công ty hoặc hợp đồng đăng ký mua cổ phần quy định một thời hạn khác ngắn hơn</t>
+          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp, Giấy xác nhận về việc thay đổi nội dung</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_giay_chung_nhan_dang_ky_doanh_nghiep`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung`.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D113_K1_E000094_HC863DA3A8CBE__234d9c7caeb7b4; RULE_LUATDN_D113_K1_E000085_HABFC666433B3__22c2142f7ac83a; RULE_LUATDN_D113_K1_E000078_H67FF516B0336__96d8cf793c1519; RULE_LUATDN_D205_K2_E000180_HA8EFB2670117__32e45121578765; RULE_LUATDN_D113_K1_E000082_H67FF516B0336__b18dfb4fdee692; RULE_LUATDN_D113_K1_E000083_H4135AC48C5CC__92ac27f8e80f5c; RULE_LUATDN_D113_K1_E000361_H9559D7A7E175__e7c07124cb07f1</t>
+          <t>RULE_ND168_D69_K8_E000307_H645CB00A88CB__1970f0cce8350d</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -8746,36 +8442,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>tach_exception_khoi_effect</t>
-        </is>
-      </c>
+      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>duoc_cap_giay_chung_nhan_dang_ky_doanh_nghiep_moi</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_k</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Được cấp Giấy chứng nhận đăng ký doanh nghiệp mới</t>
+          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp, Giấy xác nhận về việc thay đổi nội dung đăng ký doanh nghiệp, Giấy xác nhận thông báo tạm ngừng k</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_giay_chung_nhan_dang_ky_doanh_nghiep_moi`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_k`.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D30_K3_E000031_H683D2BEC0D69__9f7fb709427928</t>
+          <t>RULE_ND168_D69_K8_E000308_H645CB00A88CB__6cb2986879ea28; RULE_ND168_D69_K8_E000486_H27C3716A7863__43b7c194143b91</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -8788,36 +8480,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>duoc_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_kinh_doanh_giay_xac_nhan_thon</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Được cấp Giấy chứng nhận đăng ký hoạt động chi nhánh</t>
+          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp, Giấy xác nhận về việc thay đổi nội dung đăng ký doanh nghiệp, Giấy xác nhận thông báo tạm ngừng kinh doanh, Giấy xác nhận thôn</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_kinh_doanh_giay_xac_nhan_thon`.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D45_K3_E000041_H54A3724FA902__05e1c142b45446</t>
+          <t>RULE_ND168_D69_K8_E000487_H2A77DF79A945__61915324e2a4e1</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -8830,36 +8518,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>duoc_cap_thong_tin_duoc_luu_giu_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_va_phai_nop_phi</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_kinh_doanh_giay_xac_nhan_thong_bao_t</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Được cấp thông tin được lưu giữ trên Hệ thống thông tin quốc gia về đăng ký doanh nghiệp và phải nộp phí</t>
+          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp, Giấy xác nhận về việc thay đổi nội dung đăng ký doanh nghiệp, Giấy xác nhận thông báo tạm ngừng kinh doanh, Giấy xác nhận thông báo t</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_thong_tin_duoc_luu_giu_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep_va_phai_nop_phi`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_kinh_doanh_giay_xac_nhan_thong_bao_t`.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D33_K1_E000040_HBD0F2B965340__e0be59d28bca43</t>
+          <t>RULE_ND168_D69_K8_E000484_H27C3716A7863__9d99e90d01c504</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -8872,36 +8556,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>duoc_cap_tinh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_va_viec_khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Được cấp tỉnh cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả cho người nộp hồ sơ</t>
+          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp và việc khôi phục Giấy chứng nhận đăng ký doanh nghiệp trên Hệ thống thông tin quốc gia về đăng ký</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_tinh_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_va_viec_khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky`.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>RULE_ND168_D31_K3_E000415_HF96DE9D9BF08__715810e59d4772; RULE_ND168_D41_K2_E000425_HEEADD79DF7E1__341dcc712fe43d; RULE_ND168_D42_K2_E000430_H871CDC7A0EBD__6112b7ae8b0e38; RULE_ND168_D43_K5_E000435_HADF045408BC9__6a55deefc5885c; RULE_ND168_D44_K5_E000440_H3776FA482E45__895dd1b8852a0c</t>
+          <t>RULE_ND168_D70_K2_E000316_H76391FA4DF19__0b8d819f490a52</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -8914,78 +8594,74 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>duoc_cap_tinh_thuc_hien_quan_ly_nha_nuoc</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Được cấp tỉnh thực hiện quản lý nhà nước</t>
+          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh trong thời hạn 03 ngày làm việc kể từ ngày kết thúc thời hạn giải trình</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_tinh_thuc_hien_quan_ly_nha_nuoc`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh`.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>RULE_LUATDN_D215_K2_E000192_HA15EAD4E7536__4a0d8250bffec5</t>
+          <t>RULE_ND168_D107_K4_E000502_HAD9534ACA4E3__ff40d9db87e1fc</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>cao</t>
+          <t>trung_binh</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>tach_condition_khoi_effect</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>cap_giay</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>duoc_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Được cấp tỉnh trao giấy tiếp nhận hồ sơ và hẹn trả kết quả cho người nộp hồ sơ</t>
+          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh đồng thời ra thông báo về việc hộ kinh doanh đang làm</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `duoc_cap_tinh_trao_giay_tiep_nhan_ho_so_va_hen_tra_ket_qua_cho_nguoi_nop_ho_so`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam`.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>RULE_ND168_D31_K3_E000266_H1509A1A35C79__4bce78214f31d1; RULE_ND168_D41_K2_E000273_H906A9A038A6C__f824edde05271e; RULE_ND168_D42_K2_E000275_H821D573EEDF4__530e6c2ac4eb1f; RULE_ND168_D43_K5_E000277_H0243FD848FE3__802b6f2206ab87; RULE_ND168_D44_K5_E000279_HCA503CFECDA8__aa2d89008e4cec</t>
+          <t>RULE_ND168_D107_K8_E000327_H9246BA7D11BB__dac16f19cbbcc1; RULE_ND168_D107_K8_E000335_HE798C4D32E8B__e4edbc88f7a14a</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -8998,36 +8674,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>cap_nhat</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_dong_thoi_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_chi_nhanh_van_phong_dai</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_cap_nhat_tinh_t</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>khôi phục Giấy chứng nhận đăng ký doanh nghiệp, đồng thời cập nhật tình trạng pháp lý của doanh nghiệp, chi nhánh, văn phòng đại</t>
+          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh đồng thời ra thông báo về việc hộ kinh doanh đang làm thủ tục chấm dứt hoạt động, cập nhật tình t</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_dong_thoi_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_chi_nhanh_van_phong_dai`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_cap_nhat_tinh_t`.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>RULE_ND168_D70_K2_E000315_H76391FA4DF19__fd8923adabc565</t>
+          <t>RULE_ND168_D107_K8_E000328_H9246BA7D11BB__01bdb283d4efa8; RULE_ND168_D107_K8_E000336_HE798C4D32E8B__a51346519b4342; RULE_ND168_D107_K8_E000331_H65C05EF0DADF__a81f4623de28c9</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -9040,36 +8712,32 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>cap_nhat</t>
+          <t>thu_hoi</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_dong_thoi_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_chi_nhanh_van_phong_dai_dien_dia_diem_kinh_doanh_trong_co_so_du</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_cap_nhat_tinh_trang_phap_ly_cua_ho_kinh_doan</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>khôi phục Giấy chứng nhận đăng ký doanh nghiệp, đồng thời cập nhật tình trạng pháp lý của doanh nghiệp, chi nhánh, văn phòng đại diện, địa điểm kinh doanh trong Cơ sở dữ</t>
+          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh đồng thời ra thông báo về việc hộ kinh doanh đang làm thủ tục chấm dứt hoạt động, cập nhật tình trạng pháp lý của hộ kinh doan</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_dong_thoi_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_chi_nhanh_van_phong_dai_dien_dia_diem_kinh_doanh_trong_co_so_du`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_cap_nhat_tinh_trang_phap_ly_cua_ho_kinh_doan`.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>RULE_ND168_D70_K2_E000490_H294525A8FA40__1aeefc8cc68ed5</t>
+          <t>RULE_ND168_D107_K8_E000514_HF1DC4B5243E5__287d78470bad44</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -9082,11 +8750,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -9096,22 +8760,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_va_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_tren_cong_thong_tin_quoc_g</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp, Giấy xác nhận về việc thay đổi nội dung</t>
+          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh và thông báo về việc hộ kinh doanh đang làm thủ tục chấm dứt hoạt động trên Cổng thông tin quốc g</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_va_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_tren_cong_thong_tin_quoc_g`.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>RULE_ND168_D69_K8_E000307_H645CB00A88CB__1970f0cce8350d</t>
+          <t>RULE_ND168_D107_K8_E000329_H9246BA7D11BB__149bd3691389fa; RULE_ND168_D107_K8_E000337_HE798C4D32E8B__3fa257eb657871</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -9124,11 +8788,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9138,22 +8798,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_k</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_va_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_tren_cong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp, Giấy xác nhận về việc thay đổi nội dung đăng ký doanh nghiệp, Giấy xác nhận thông báo tạm ngừng k</t>
+          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh và thông báo về việc hộ kinh doanh đang làm thủ tục chấm dứt hoạt động trên Cổng thông tin quốc gia về đăng ký doanh nghiệp</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_k`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_va_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_tren_cong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep`.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>RULE_ND168_D69_K8_E000308_H645CB00A88CB__6cb2986879ea28; RULE_ND168_D69_K8_E000486_H27C3716A7863__43b7c194143b91</t>
+          <t>RULE_ND168_D107_K8_E000504_HE6BBDAF42D70__3340ce83b0c5f4</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -9166,11 +8826,7 @@
           <t>cao</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9180,413 +8836,35 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_kinh_doanh_giay_xac_nhan_thon</t>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh_van_phong_dai_dien</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp, Giấy xác nhận về việc thay đổi nội dung đăng ký doanh nghiệp, Giấy xác nhận thông báo tạm ngừng kinh doanh, Giấy xác nhận thôn</t>
+          <t>thu hồi Giấy chứng nhận đăng ký hoạt động chi nhánh, văn phòng đại diện trong thời hạn 03 ngày làm việc kể từ ngày kết thúc thời hạn giải trình</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_kinh_doanh_giay_xac_nhan_thon`.</t>
+          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh_van_phong_dai_dien`.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>RULE_ND168_D69_K8_E000487_H2A77DF79A945__61915324e2a4e1</t>
+          <t>RULE_ND168_D71_K3_E000496_HD4B75A6952A5__ca660bf58d6b4b</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>khong</t>
+          <t>co</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>cao</t>
+          <t>trung_binh</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>thu_hoi</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_kinh_doanh_giay_xac_nhan_thong_bao_t</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp, Giấy xác nhận về việc thay đổi nội dung đăng ký doanh nghiệp, Giấy xác nhận thông báo tạm ngừng kinh doanh, Giấy xác nhận thông báo t</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_giay_xac_nhan_ve_viec_thay_doi_noi_dung_dang_ky_doanh_nghiep_giay_xac_nhan_thong_bao_tam_ngung_kinh_doanh_giay_xac_nhan_thong_bao_t`.</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>RULE_ND168_D69_K8_E000484_H27C3716A7863__9d99e90d01c504</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>cao</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>thu_hoi</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_va_viec_khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>thu hồi Giấy chứng nhận đăng ký doanh nghiệp và việc khôi phục Giấy chứng nhận đăng ký doanh nghiệp trên Hệ thống thông tin quốc gia về đăng ký</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_doanh_nghiep_va_viec_khoi_phuc_giay_chung_nhan_dang_ky_doanh_nghiep_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky`.</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>RULE_ND168_D70_K2_E000316_H76391FA4DF19__0b8d819f490a52</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>cao</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>thu_hoi</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh trong thời hạn 03 ngày làm việc kể từ ngày kết thúc thời hạn giải trình</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh`.</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>RULE_ND168_D107_K4_E000502_HAD9534ACA4E3__ff40d9db87e1fc</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>co</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>trung_binh</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>tach_condition_khoi_effect</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>thu_hoi</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh đồng thời ra thông báo về việc hộ kinh doanh đang làm</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam`.</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>RULE_ND168_D107_K8_E000327_H9246BA7D11BB__dac16f19cbbcc1; RULE_ND168_D107_K8_E000335_HE798C4D32E8B__e4edbc88f7a14a</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>cao</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>thu_hoi</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_cap_nhat_tinh_t</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh đồng thời ra thông báo về việc hộ kinh doanh đang làm thủ tục chấm dứt hoạt động, cập nhật tình t</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_cap_nhat_tinh_t`.</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>RULE_ND168_D107_K8_E000328_H9246BA7D11BB__01bdb283d4efa8; RULE_ND168_D107_K8_E000336_HE798C4D32E8B__a51346519b4342; RULE_ND168_D107_K8_E000331_H65C05EF0DADF__a81f4623de28c9</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>cao</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>thu_hoi</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_cap_nhat_tinh_trang_phap_ly_cua_ho_kinh_doan</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh đồng thời ra thông báo về việc hộ kinh doanh đang làm thủ tục chấm dứt hoạt động, cập nhật tình trạng pháp lý của hộ kinh doan</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_dong_thoi_ra_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_cap_nhat_tinh_trang_phap_ly_cua_ho_kinh_doan`.</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>RULE_ND168_D107_K8_E000514_HF1DC4B5243E5__287d78470bad44</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>cao</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>thu_hoi</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_va_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_tren_cong_thong_tin_quoc_g</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh và thông báo về việc hộ kinh doanh đang làm thủ tục chấm dứt hoạt động trên Cổng thông tin quốc g</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_va_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_tren_cong_thong_tin_quoc_g`.</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>RULE_ND168_D107_K8_E000329_H9246BA7D11BB__149bd3691389fa; RULE_ND168_D107_K8_E000337_HE798C4D32E8B__3fa257eb657871</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>cao</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>thu_hoi</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_va_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_tren_cong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh và thông báo về việc hộ kinh doanh đang làm thủ tục chấm dứt hoạt động trên Cổng thông tin quốc gia về đăng ký doanh nghiệp</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_va_thong_bao_ve_viec_ho_kinh_doanh_dang_lam_thu_tuc_cham_dut_hoat_dong_tren_cong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep`.</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>RULE_ND168_D107_K8_E000504_HE6BBDAF42D70__3340ce83b0c5f4</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>khong</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>cao</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>thu_hoi</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>thu_hoi_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh_van_phong_dai_dien</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>thu hồi Giấy chứng nhận đăng ký hoạt động chi nhánh, văn phòng đại diện trong thời hạn 03 ngày làm việc kể từ ngày kết thúc thời hạn giải trình</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Kết quả/hậu quả (đã tách điều kiện/ngoại lệ nếu có). `thu_hoi_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh_van_phong_dai_dien`.</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>RULE_ND168_D71_K3_E000496_HD4B75A6952A5__ca660bf58d6b4b</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>co</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>trung_binh</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
         <is>
           <t>tach_condition_khoi_effect</t>
         </is>
@@ -11791,7 +11069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11831,6 +11109,632 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>exception</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>effect_vocabulary</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>duoc_cap_giay_chung_nhan_dang_ky_doanh_nghiep_tru_truong_hop_dieu_le_cong_ty_hoac_hop_dong_dang_ky_mua_co_phan_quy_dinh_mot_thoi_han_khac_ngan_hon</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>tru_truong_hop_dieu_le_cong_ty_hoac_hop_dong_dang_ky_mua_co_phan_quy_dinh_mot_thoi_han_khac_ngan_hon</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>được cấp Giấy chứng nhận đăng ký doanh nghiệp, trừ trường hợp Điều lệ công ty hoặc hợp đồng đăng ký mua cổ phần quy định một thời hạn khác ngắn hơn</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>tach_exception_condition_khoi_effect</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>RULE_LUATDN_D113_K1_E000082_H67FF516B0336__b18dfb4fdee692; RULE_LUATDN_D113_K1_E000083_H4135AC48C5CC__92ac27f8e80f5c; RULE_LUATDN_D113_K1_E000361_H9559D7A7E175__e7c07124cb07f1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>exception</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>effect_vocabulary</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>chap_thuan_tru_truong_hop_hoi_dong_thanh_vien_quyet_dinh_thoi_han_khac</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>tru_truong_hop_hoi_dong_thanh_vien_quyet_dinh_thoi_han_khac</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>chấp thuận, trừ trường hợp Hội đồng thành viên quyết định thời hạn khác</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>tach_exception_condition_khoi_effect</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>RULE_LUATDN_D186_K2_E000128_H978952EE6FD4__271a076b3bf9cb; RULE_LUATDN_D186_K2_E000364_HC305BFE2E363__e1e8bea05ff736; RULE_LUATDN_D186_K2_E000125_H2FC30FD46A92__59df9f03b09822</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>effect_vocabulary</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>cap_giay_chung_nhan_dang_ky_doanh_nghiep_neu_co_du_dieu_kien_quy_dinh_tai_khoan_1_dieu_nay_va_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_tren_co_so_du_lieu_quoc_gia_ve</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>neu_co_du_dieu_kien_quy_dinh_tai_khoan_1_dieu_nay_va_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_tren_co_so_du_lieu_quoc_gia_ve</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>cấp Giấy chứng nhận đăng ký doanh nghiệp nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>tach_exception_condition_khoi_effect</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>RULE_LUATDN_D205_K2_E000171_HC103AB968CE3__db7af93bea0162</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>effect_vocabulary</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>cap_giay_chung_nhan_dang_ky_doanh_nghiep_neu_co_du_dieu_kien_quy_dinh_tai_khoan_1_dieu_nay_va_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_tren_co_so_du_lieu_quoc_gia_ve_dang_ky_doanh_nghie</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>neu_co_du_dieu_kien_quy_dinh_tai_khoan_1_dieu_nay_va_cap_nhat_tinh_trang_phap_ly_cua_doanh_nghiep_tren_co_so_du_lieu_quoc_gia_ve_dang_ky_doanh_nghie</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>cấp Giấy chứng nhận đăng ký doanh nghiệp nếu có đủ điều kiện quy định tại khoản 1 Điều này và cập nhật tình trạng pháp lý của doanh nghiệp trên Cơ sở dữ liệu quốc gia về đăng ký doanh nghiệ</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>tach_exception_condition_khoi_effect</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>RULE_LUATDN_D205_K2_E000376_HDE4D11047D02__d8fcb45eefe40d</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>effect_vocabulary</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>cap_giay_chung_nhan_dang_ky_doanh_nghiep_neu_co_du_dieu_kien_quy</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>neu_co_du_dieu_kien_quy</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>cấp Giấy chứng nhận đăng ký doanh nghiệp nếu có đủ điều kiện quy</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>tach_exception_condition_khoi_effect</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>RULE_LUATDN_D205_K2_E000174_HBB868040B12A__747ded761e8875</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>effect_vocabulary</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_ho_kinh_doanh_trong_thoi_han_03_ngay_lam_viec_ke_tu_ngay_ket_thuc_thoi_han_giai_trinh</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>trong_thoi_han_03_ngay_lam_viec_ke_tu_ngay_ket_thuc_thoi_han_giai_trinh</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>thu hồi Giấy chứng nhận đăng ký hộ kinh doanh trong thời hạn 03 ngày làm việc kể từ ngày kết thúc thời hạn giải trình</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>tach_exception_condition_khoi_effect</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>RULE_ND168_D107_K4_E000502_HAD9534ACA4E3__ff40d9db87e1fc</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>effect_vocabulary</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>cham_dut_hoat_dong_doi_voi_chi_nhanh_van_phong_dai_dien_dia_diem_kinh_doanh</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>doi_voi_chi_nhanh_van_phong_dai_dien_dia_diem_kinh_doanh</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>chấm dứt hoạt động đối với chi nhánh, văn phòng đại diện, địa điểm kinh doanh</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>tach_exception_condition_khoi_effect</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>RULE_ND168_D118_K3_E000522_H0811C24751E0__7fb44d85940b04; RULE_ND168_D118_K3_E000341_H6839229D9C6F__6f008278ee22c6</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>effect_vocabulary</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>thu_hoi_giay_chung_nhan_dang_ky_hoat_dong_chi_nhanh_van_phong_dai_dien_trong_thoi_han_03_ngay_lam_viec_ke_tu_ngay_ket_thuc_thoi_han_giai_trinh</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>trong_thoi_han_03_ngay_lam_viec_ke_tu_ngay_ket_thuc_thoi_han_giai_trinh</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>thu hồi Giấy chứng nhận đăng ký hoạt động chi nhánh, văn phòng đại diện trong thời hạn 03 ngày làm việc kể từ ngày kết thúc thời hạn giải trình</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>tach_exception_condition_khoi_effect</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>RULE_ND168_D71_K3_E000496_HD4B75A6952A5__ca660bf58d6b4b</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>discourse_or_condition</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>object_vocabulary</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>phai_co_cac_giay_to_sau_day</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>phải có các giấy tờ sau đây | phải có các giấy tờ sau đây:</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>loai_condition_hoac_scope_khoi_object</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>RULE_ND168_D28_K7_E000248_H189EC3F188B6__506b814bf616a9; RULE_ND168_D28_K7_E000410_HAB891EF8FB58__9c53376c4e0d7b; RULE_ND168_D28_K7_E000409_HAB891EF8FB58__b4611058cb4d7c; RULE_ND168_D28_K7_E000411_HAB891EF8FB58__9271c5cad72e01</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>discourse_or_condition</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>object_vocabulary</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>khi_dang_ky_thanh_lap_doanh_nghiep</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>khi đăng ký thành lập doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>loai_condition_hoac_scope_khoi_object</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>RULE_LUATDN_D120_K2_E000110_H2F74D053E9ED__e3455c07586f9b; RULE_LUATDN_D120_K2_E000106_H50EB455F10E0__d9e773edb1f1e0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>discourse_or_condition</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>object_vocabulary</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>khi_trinh_dai_hoi_dong_co_dong_xem_xet</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>khi trình Đại hội đồng cổ đông xem xét</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>loai_condition_hoac_scope_khoi_object</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>RULE_LUATDN_D175_K2_E000122_H3A810D8013F8__cecb075395e7d9</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>discourse_or_condition</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>object_vocabulary</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>hop_dong_da_ky_voi_khach_hang_va_nguoi_lao_dong</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>hợp đồng đã ký với khách hàng và người lao động</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>loai_condition_hoac_scope_khoi_object</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>RULE_LUATDN_D206_K3_E000183_HB3760B0CD551__fa214a6f1d0709</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>discourse_or_condition</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>object_vocabulary</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>tru_truong_hop_doanh_nghiep</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>trừ trường hợp doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>loai_condition_hoac_scope_khoi_object</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>RULE_LUATDN_D206_K3_E000184_HB3760B0CD551__d9cc7b2a45cf2a</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>discourse_or_condition</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>object_vocabulary</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>hop_dong_da_ky_voi_khach_hang_va_nguoi_lao_dong_tru_truong_hop_doanh_nghiep_chu_no_khach_hang_va_nguoi</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>hợp đồng đã ký với khách hàng và người lao động, trừ trường hợp doanh nghiệp, chủ nợ, khách hàng và người</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>loai_condition_hoac_scope_khoi_object</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>RULE_LUATDN_D206_K3_E000182_HB3760B0CD551__0c3013b06a8c7b</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>discourse_or_condition</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>object_vocabulary</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>khi_thay_doi_noi_dung_giay_chung_nhan_dang_ky_doanh_nghiep_quy_dinh_tai_dieu_28_cua_luat_nay</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>khi thay đổi nội dung Giấy chứng nhận đăng ký doanh nghiệp quy định tại Điều 28 của Luật này</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>loai_condition_hoac_scope_khoi_object</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>RULE_LUATDN_D30_K1_E000020_H4E002511683E__bc79ef05e292ad</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>discourse_or_condition</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>object_vocabulary</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>khi_ho_so_dang_ky_doanh_nghiep_chua_duoc_chap_thuan_tren_he_thong_thong_tin_quoc_gia_ve_dang_ky_doanh_nghiep</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>khi hồ sơ đăng ký doanh nghiệp chưa được chấp thuận trên Hệ thống thông tin quốc gia về đăng ký doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>loai_condition_hoac_scope_khoi_object</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>RULE_ND168_D31_K6_E000267_H565D1BB5E0AC__243ed69455d8ce; RULE_ND168_D31_K6_E000271_H565D1BB5E0AC__515f331279a5a7; RULE_ND168_D31_K6_E000416_HF58B712D1CE4__7867763b848ee0; RULE_ND168_D31_K6_E000419_H46A4A566E7A4__38e6cb2ba88b0e; RULE_ND168_D31_K6_E000421_H46A4A566E7A4__0907921944a235</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>discourse_or_condition</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>object_vocabulary</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>truong_hop_doanh_nghiep_cap_nhat</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>trường hợp doanh nghiệp cập nhật</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>loai_condition_hoac_scope_khoi_object</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>RULE_ND168_D57_K3_E000299_HA471205F1C6F__44c27f4eae6de3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>discourse_or_condition</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>object_vocabulary</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>van_ban_giai_trinh_cua_doanh_nghiep_ve_ly_do_dang_ky_thay_doi_kem_ho_so_dang_ky_thay_doi_khi_dang_ky_phuc_vu_giai_the</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>văn bản giải trình của doanh nghiệp về lý do đăng ký thay đổi (kèm hồ sơ đăng ký thay đổi khi đăng ký phục vụ giải thể)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>loai_condition_hoac_scope_khoi_object</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>RULE_ND168_D59_K2_B_E000479_H6CE5F7A93C8B__e80d74b1b90e68; RULE_ND168_D59_K2_B_E000480_H6CE5F7A93C8B__56e9128f42f85d</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>